<commit_message>
feat(deploy): update database schema, admin registry, and production deployment configuration
</commit_message>
<xml_diff>
--- a/data/private/admin_registry.xlsx
+++ b/data/private/admin_registry.xlsx
@@ -548,7 +548,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 13:48:24</t>
+          <t>2026-08-30 15:45:24</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -639,7 +639,7 @@
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="2" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -663,12 +663,12 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>13:48:34</t>
+          <t>15:45:48</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 13:48:34</t>
+          <t>2026-08-30 15:45:49</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -679,7 +679,7 @@
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="2" t="n">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
@@ -703,12 +703,12 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>13:48:20</t>
+          <t>15:45:21</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 13:48:20</t>
+          <t>2026-08-30 15:45:22</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add cloud-compatible browser camera attendance
</commit_message>
<xml_diff>
--- a/data/private/admin_registry.xlsx
+++ b/data/private/admin_registry.xlsx
@@ -548,7 +548,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 15:45:24</t>
+          <t>2026-08-30 16:40:22</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -639,7 +639,7 @@
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="2" t="n">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -663,12 +663,12 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>15:45:48</t>
+          <t>16:40:33</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 15:45:49</t>
+          <t>2026-08-30 16:40:34</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -679,7 +679,7 @@
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="2" t="n">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
@@ -703,12 +703,12 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>15:45:21</t>
+          <t>16:40:19</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 15:45:22</t>
+          <t>2026-08-30 16:40:19</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">

</xml_diff>